<commit_message>
Refactor e_ik_cmf function to streamline data extraction from CMF files
- Removed the option to suppress warnings during type conversion.
- Simplified the data reading process by forcing all columns to text format.
- Consolidated the data processing logic to improve readability and maintainability.
- Updated the return value to directly return the processed data frame.
- Adjusted the handling of metadata and column renaming for consistency.
- Updated the handling of monetary and date conversions for better accuracy.
- Modified the logic for creating derived columns such as 'empresa' and 'conta.interno'.
- Updated the documentation to reflect the changes in function parameters and behavior.

Updated several Excel files in the 'dados' directory to ensure compatibility with the new function implementation.
</commit_message>
<xml_diff>
--- a/dados/Estação - Repasse PF e PJ.xlsx
+++ b/dados/Estação - Repasse PF e PJ.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://incorporadoraampla-my.sharepoint.com/personal/vitor_amplaincorporadora_com_br/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://incorporadoraampla.sharepoint.com/sites/Controladoria/Documentos Compartilhados/amplaGitHub/dados/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="36" documentId="8_{3456AD2F-C159-4FF2-95DE-59A3AA000877}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{512B443C-0B4E-4BEE-915D-3D0904C56B66}"/>
+  <xr:revisionPtr revIDLastSave="38" documentId="8_{3456AD2F-C159-4FF2-95DE-59A3AA000877}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6E1774D7-7728-441C-B15E-E2B9A1187D2E}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-11640" windowWidth="20640" windowHeight="11160" xr2:uid="{DE446C1C-D0AB-4EA1-8007-02302B937BC4}"/>
+    <workbookView xWindow="-57600" yWindow="-3555" windowWidth="14445" windowHeight="15600" xr2:uid="{DE446C1C-D0AB-4EA1-8007-02302B937BC4}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -723,14 +723,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="165" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
@@ -790,48 +789,6 @@
         </top>
         <bottom/>
       </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="0"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4"/>
-          <bgColor theme="4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
     </dxf>
     <dxf>
       <font>
@@ -1292,6 +1249,48 @@
         </top>
       </border>
     </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1306,25 +1305,25 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5E07FEE3-FE59-43C8-862A-29C8248948D4}" name="Tabela1" displayName="Tabela1" ref="A1:R285" totalsRowShown="0" headerRowDxfId="2" dataDxfId="3" tableBorderDxfId="20">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5E07FEE3-FE59-43C8-862A-29C8248948D4}" name="Tabela1" displayName="Tabela1" ref="A1:R285" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19" tableBorderDxfId="18">
   <autoFilter ref="A1:R285" xr:uid="{5E07FEE3-FE59-43C8-862A-29C8248948D4}"/>
   <tableColumns count="18">
-    <tableColumn id="1" xr3:uid="{84208E7C-F8E1-401F-84A5-228777D2F120}" name="data.movimento" dataDxfId="19"/>
-    <tableColumn id="2" xr3:uid="{1259D875-A5F6-405F-8B68-52570D64152A}" name="documento" dataDxfId="18"/>
-    <tableColumn id="3" xr3:uid="{182C9E41-C31F-4CC3-9452-F79AECAFAFD8}" name="descricao" dataDxfId="17"/>
-    <tableColumn id="4" xr3:uid="{2E1A0E32-8FDB-4C0A-A0A4-595A455E6BCF}" name="valor" dataDxfId="16"/>
-    <tableColumn id="5" xr3:uid="{6E9EA891-1600-4522-AFC9-6C1B31FD5EFD}" name="saldo" dataDxfId="15"/>
-    <tableColumn id="6" xr3:uid="{98855389-D664-407D-AEF5-B18912153014}" name="repasse" dataDxfId="14"/>
-    <tableColumn id="7" xr3:uid="{63F64382-EE14-4F2B-AA0C-9981892B8652}" name="pj" dataDxfId="13"/>
-    <tableColumn id="8" xr3:uid="{D3646397-CDA1-450F-BD34-C0F0AD21D756}" name="conta.interno" dataDxfId="12"/>
-    <tableColumn id="9" xr3:uid="{71485BA4-5C04-497D-84E8-EC053AADD306}" name="conta" dataDxfId="11"/>
-    <tableColumn id="10" xr3:uid="{95232551-3708-420B-AAE6-E31680AEFE20}" name="agencia" dataDxfId="10"/>
-    <tableColumn id="11" xr3:uid="{B7D68A0A-928F-438D-9F50-EAEF26204137}" name="produto" dataDxfId="9"/>
-    <tableColumn id="12" xr3:uid="{ABA3FE27-6A55-47C4-9451-B018E5578621}" name="cnpj" dataDxfId="8"/>
-    <tableColumn id="13" xr3:uid="{B3FEFFE2-497A-4D07-8C1F-D0814E259433}" name="empreendimento" dataDxfId="7"/>
-    <tableColumn id="14" xr3:uid="{963A342F-A243-4C73-A38A-09F71952D400}" name="periodo.inicio" dataDxfId="6"/>
-    <tableColumn id="15" xr3:uid="{1B315A5E-FF27-4654-93DB-C5EE8BAE9611}" name="periodo.fim" dataDxfId="5"/>
-    <tableColumn id="16" xr3:uid="{3B643482-09B2-4150-92A6-24FBB9A564BA}" name="data.consulta" dataDxfId="4"/>
+    <tableColumn id="1" xr3:uid="{84208E7C-F8E1-401F-84A5-228777D2F120}" name="data.movimento" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{1259D875-A5F6-405F-8B68-52570D64152A}" name="documento" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{182C9E41-C31F-4CC3-9452-F79AECAFAFD8}" name="descricao" dataDxfId="15"/>
+    <tableColumn id="4" xr3:uid="{2E1A0E32-8FDB-4C0A-A0A4-595A455E6BCF}" name="valor" dataDxfId="14"/>
+    <tableColumn id="5" xr3:uid="{6E9EA891-1600-4522-AFC9-6C1B31FD5EFD}" name="saldo" dataDxfId="13"/>
+    <tableColumn id="6" xr3:uid="{98855389-D664-407D-AEF5-B18912153014}" name="repasse" dataDxfId="12"/>
+    <tableColumn id="7" xr3:uid="{63F64382-EE14-4F2B-AA0C-9981892B8652}" name="pj" dataDxfId="11"/>
+    <tableColumn id="8" xr3:uid="{D3646397-CDA1-450F-BD34-C0F0AD21D756}" name="conta.interno" dataDxfId="10"/>
+    <tableColumn id="9" xr3:uid="{71485BA4-5C04-497D-84E8-EC053AADD306}" name="conta" dataDxfId="9"/>
+    <tableColumn id="10" xr3:uid="{95232551-3708-420B-AAE6-E31680AEFE20}" name="agencia" dataDxfId="8"/>
+    <tableColumn id="11" xr3:uid="{B7D68A0A-928F-438D-9F50-EAEF26204137}" name="produto" dataDxfId="7"/>
+    <tableColumn id="12" xr3:uid="{ABA3FE27-6A55-47C4-9451-B018E5578621}" name="cnpj" dataDxfId="6"/>
+    <tableColumn id="13" xr3:uid="{B3FEFFE2-497A-4D07-8C1F-D0814E259433}" name="empreendimento" dataDxfId="5"/>
+    <tableColumn id="14" xr3:uid="{963A342F-A243-4C73-A38A-09F71952D400}" name="periodo.inicio" dataDxfId="4"/>
+    <tableColumn id="15" xr3:uid="{1B315A5E-FF27-4654-93DB-C5EE8BAE9611}" name="periodo.fim" dataDxfId="3"/>
+    <tableColumn id="16" xr3:uid="{3B643482-09B2-4150-92A6-24FBB9A564BA}" name="data.consulta" dataDxfId="2"/>
     <tableColumn id="17" xr3:uid="{7C379743-A2C5-4A42-9969-BD5494438747}" name="contrato.6" dataDxfId="1"/>
     <tableColumn id="18" xr3:uid="{34A8CF0A-03D2-4368-975F-BABD054EBCF0}" name="arquivo" dataDxfId="0"/>
   </tableColumns>
@@ -1684,10 +1683,10 @@
       <c r="E1" s="4" t="s">
         <v>186</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="5" t="s">
         <v>188</v>
       </c>
       <c r="H1" s="4" t="s">
@@ -1774,7 +1773,7 @@
       <c r="Q2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="R2" s="5" t="s">
+      <c r="R2" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1828,7 +1827,7 @@
       <c r="Q3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="R3" s="5" t="s">
+      <c r="R3" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1882,7 +1881,7 @@
       <c r="Q4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="R4" s="5" t="s">
+      <c r="R4" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1936,7 +1935,7 @@
       <c r="Q5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="R5" s="5" t="s">
+      <c r="R5" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1990,7 +1989,7 @@
       <c r="Q6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="R6" s="5" t="s">
+      <c r="R6" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2044,7 +2043,7 @@
       <c r="Q7" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="R7" s="5" t="s">
+      <c r="R7" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2098,7 +2097,7 @@
       <c r="Q8" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="R8" s="5" t="s">
+      <c r="R8" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2152,7 +2151,7 @@
       <c r="Q9" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="R9" s="5" t="s">
+      <c r="R9" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2206,7 +2205,7 @@
       <c r="Q10" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="R10" s="5" t="s">
+      <c r="R10" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2260,7 +2259,7 @@
       <c r="Q11" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="R11" s="5" t="s">
+      <c r="R11" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2314,7 +2313,7 @@
       <c r="Q12" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="R12" s="5" t="s">
+      <c r="R12" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2368,7 +2367,7 @@
       <c r="Q13" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="R13" s="5" t="s">
+      <c r="R13" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2422,7 +2421,7 @@
       <c r="Q14" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="R14" s="5" t="s">
+      <c r="R14" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2476,7 +2475,7 @@
       <c r="Q15" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="R15" s="5" t="s">
+      <c r="R15" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2530,7 +2529,7 @@
       <c r="Q16" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="R16" s="5" t="s">
+      <c r="R16" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2584,7 +2583,7 @@
       <c r="Q17" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="R17" s="5" t="s">
+      <c r="R17" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2638,7 +2637,7 @@
       <c r="Q18" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="R18" s="5" t="s">
+      <c r="R18" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2692,7 +2691,7 @@
       <c r="Q19" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="R19" s="5" t="s">
+      <c r="R19" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2746,7 +2745,7 @@
       <c r="Q20" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="R20" s="5" t="s">
+      <c r="R20" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2800,7 +2799,7 @@
       <c r="Q21" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="R21" s="5" t="s">
+      <c r="R21" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2854,7 +2853,7 @@
       <c r="Q22" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R22" s="5" t="s">
+      <c r="R22" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2908,7 +2907,7 @@
       <c r="Q23" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="R23" s="5" t="s">
+      <c r="R23" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2962,7 +2961,7 @@
       <c r="Q24" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="R24" s="5" t="s">
+      <c r="R24" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3016,7 +3015,7 @@
       <c r="Q25" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="R25" s="5" t="s">
+      <c r="R25" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3070,7 +3069,7 @@
       <c r="Q26" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="R26" s="5" t="s">
+      <c r="R26" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3124,7 +3123,7 @@
       <c r="Q27" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="R27" s="5" t="s">
+      <c r="R27" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3178,7 +3177,7 @@
       <c r="Q28" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="R28" s="5" t="s">
+      <c r="R28" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3232,7 +3231,7 @@
       <c r="Q29" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="R29" s="5" t="s">
+      <c r="R29" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3286,7 +3285,7 @@
       <c r="Q30" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="R30" s="5" t="s">
+      <c r="R30" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3340,7 +3339,7 @@
       <c r="Q31" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="R31" s="5" t="s">
+      <c r="R31" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3394,7 +3393,7 @@
       <c r="Q32" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="R32" s="5" t="s">
+      <c r="R32" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3448,7 +3447,7 @@
       <c r="Q33" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="R33" s="5" t="s">
+      <c r="R33" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3502,7 +3501,7 @@
       <c r="Q34" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="R34" s="5" t="s">
+      <c r="R34" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3556,7 +3555,7 @@
       <c r="Q35" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="R35" s="5" t="s">
+      <c r="R35" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3610,7 +3609,7 @@
       <c r="Q36" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="R36" s="5" t="s">
+      <c r="R36" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3664,7 +3663,7 @@
       <c r="Q37" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="R37" s="5" t="s">
+      <c r="R37" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3718,7 +3717,7 @@
       <c r="Q38" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="R38" s="5" t="s">
+      <c r="R38" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3772,7 +3771,7 @@
       <c r="Q39" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="R39" s="5" t="s">
+      <c r="R39" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3826,7 +3825,7 @@
       <c r="Q40" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="R40" s="5" t="s">
+      <c r="R40" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3880,7 +3879,7 @@
       <c r="Q41" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="R41" s="5" t="s">
+      <c r="R41" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3934,7 +3933,7 @@
       <c r="Q42" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="R42" s="5" t="s">
+      <c r="R42" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3988,7 +3987,7 @@
       <c r="Q43" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="R43" s="5" t="s">
+      <c r="R43" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -4042,7 +4041,7 @@
       <c r="Q44" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="R44" s="5" t="s">
+      <c r="R44" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -4096,7 +4095,7 @@
       <c r="Q45" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="R45" s="5" t="s">
+      <c r="R45" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -4150,7 +4149,7 @@
       <c r="Q46" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="R46" s="5" t="s">
+      <c r="R46" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -4204,7 +4203,7 @@
       <c r="Q47" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="R47" s="5" t="s">
+      <c r="R47" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -4258,7 +4257,7 @@
       <c r="Q48" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="R48" s="5" t="s">
+      <c r="R48" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -4312,7 +4311,7 @@
       <c r="Q49" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="R49" s="5" t="s">
+      <c r="R49" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -4366,7 +4365,7 @@
       <c r="Q50" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="R50" s="5" t="s">
+      <c r="R50" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -4420,7 +4419,7 @@
       <c r="Q51" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="R51" s="5" t="s">
+      <c r="R51" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -4474,7 +4473,7 @@
       <c r="Q52" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="R52" s="5" t="s">
+      <c r="R52" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -4528,7 +4527,7 @@
       <c r="Q53" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="R53" s="5" t="s">
+      <c r="R53" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -4582,7 +4581,7 @@
       <c r="Q54" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="R54" s="5" t="s">
+      <c r="R54" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -4636,7 +4635,7 @@
       <c r="Q55" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="R55" s="5" t="s">
+      <c r="R55" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -4690,7 +4689,7 @@
       <c r="Q56" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="R56" s="5" t="s">
+      <c r="R56" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -4744,7 +4743,7 @@
       <c r="Q57" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="R57" s="5" t="s">
+      <c r="R57" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -4798,7 +4797,7 @@
       <c r="Q58" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="R58" s="5" t="s">
+      <c r="R58" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -4852,7 +4851,7 @@
       <c r="Q59" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="R59" s="5" t="s">
+      <c r="R59" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -4906,7 +4905,7 @@
       <c r="Q60" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="R60" s="5" t="s">
+      <c r="R60" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -4960,7 +4959,7 @@
       <c r="Q61" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="R61" s="5" t="s">
+      <c r="R61" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -5014,7 +5013,7 @@
       <c r="Q62" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="R62" s="5" t="s">
+      <c r="R62" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -5068,7 +5067,7 @@
       <c r="Q63" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="R63" s="5" t="s">
+      <c r="R63" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -5122,7 +5121,7 @@
       <c r="Q64" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="R64" s="5" t="s">
+      <c r="R64" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -5176,7 +5175,7 @@
       <c r="Q65" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="R65" s="5" t="s">
+      <c r="R65" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -5230,7 +5229,7 @@
       <c r="Q66" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="R66" s="5" t="s">
+      <c r="R66" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -5284,7 +5283,7 @@
       <c r="Q67" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="R67" s="5" t="s">
+      <c r="R67" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -5338,7 +5337,7 @@
       <c r="Q68" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="R68" s="5" t="s">
+      <c r="R68" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -5392,7 +5391,7 @@
       <c r="Q69" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="R69" s="5" t="s">
+      <c r="R69" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -5446,7 +5445,7 @@
       <c r="Q70" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="R70" s="5" t="s">
+      <c r="R70" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -5500,7 +5499,7 @@
       <c r="Q71" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="R71" s="5" t="s">
+      <c r="R71" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -5554,7 +5553,7 @@
       <c r="Q72" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="R72" s="5" t="s">
+      <c r="R72" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -5608,7 +5607,7 @@
       <c r="Q73" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="R73" s="5" t="s">
+      <c r="R73" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -5662,7 +5661,7 @@
       <c r="Q74" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="R74" s="5" t="s">
+      <c r="R74" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -5716,7 +5715,7 @@
       <c r="Q75" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="R75" s="5" t="s">
+      <c r="R75" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -5770,7 +5769,7 @@
       <c r="Q76" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="R76" s="5" t="s">
+      <c r="R76" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -5824,7 +5823,7 @@
       <c r="Q77" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="R77" s="5" t="s">
+      <c r="R77" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -5878,7 +5877,7 @@
       <c r="Q78" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="R78" s="5" t="s">
+      <c r="R78" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -5932,7 +5931,7 @@
       <c r="Q79" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="R79" s="5" t="s">
+      <c r="R79" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -5986,7 +5985,7 @@
       <c r="Q80" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="R80" s="5" t="s">
+      <c r="R80" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -6040,7 +6039,7 @@
       <c r="Q81" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="R81" s="5" t="s">
+      <c r="R81" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -6094,7 +6093,7 @@
       <c r="Q82" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="R82" s="5" t="s">
+      <c r="R82" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -6148,7 +6147,7 @@
       <c r="Q83" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="R83" s="5" t="s">
+      <c r="R83" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -6202,7 +6201,7 @@
       <c r="Q84" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="R84" s="5" t="s">
+      <c r="R84" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -6256,7 +6255,7 @@
       <c r="Q85" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="R85" s="5" t="s">
+      <c r="R85" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -6310,7 +6309,7 @@
       <c r="Q86" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="R86" s="5" t="s">
+      <c r="R86" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -6364,7 +6363,7 @@
       <c r="Q87" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="R87" s="5" t="s">
+      <c r="R87" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -6418,7 +6417,7 @@
       <c r="Q88" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="R88" s="5" t="s">
+      <c r="R88" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -6472,7 +6471,7 @@
       <c r="Q89" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="R89" s="5" t="s">
+      <c r="R89" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -6526,7 +6525,7 @@
       <c r="Q90" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="R90" s="5" t="s">
+      <c r="R90" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -6580,7 +6579,7 @@
       <c r="Q91" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="R91" s="5" t="s">
+      <c r="R91" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -6634,7 +6633,7 @@
       <c r="Q92" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="R92" s="5" t="s">
+      <c r="R92" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -6688,7 +6687,7 @@
       <c r="Q93" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="R93" s="5" t="s">
+      <c r="R93" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -6742,7 +6741,7 @@
       <c r="Q94" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="R94" s="5" t="s">
+      <c r="R94" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -6796,7 +6795,7 @@
       <c r="Q95" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="R95" s="5" t="s">
+      <c r="R95" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -6850,7 +6849,7 @@
       <c r="Q96" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="R96" s="5" t="s">
+      <c r="R96" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -6904,7 +6903,7 @@
       <c r="Q97" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="R97" s="5" t="s">
+      <c r="R97" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -6958,7 +6957,7 @@
       <c r="Q98" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="R98" s="5" t="s">
+      <c r="R98" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -7012,7 +7011,7 @@
       <c r="Q99" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="R99" s="5" t="s">
+      <c r="R99" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -7066,7 +7065,7 @@
       <c r="Q100" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="R100" s="5" t="s">
+      <c r="R100" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -7120,7 +7119,7 @@
       <c r="Q101" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="R101" s="5" t="s">
+      <c r="R101" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -7174,7 +7173,7 @@
       <c r="Q102" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="R102" s="5" t="s">
+      <c r="R102" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -7228,7 +7227,7 @@
       <c r="Q103" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="R103" s="5" t="s">
+      <c r="R103" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -7282,7 +7281,7 @@
       <c r="Q104" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="R104" s="5" t="s">
+      <c r="R104" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -7336,7 +7335,7 @@
       <c r="Q105" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="R105" s="5" t="s">
+      <c r="R105" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -7390,7 +7389,7 @@
       <c r="Q106" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="R106" s="5" t="s">
+      <c r="R106" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -7444,7 +7443,7 @@
       <c r="Q107" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="R107" s="5" t="s">
+      <c r="R107" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -7498,7 +7497,7 @@
       <c r="Q108" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="R108" s="5" t="s">
+      <c r="R108" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -7552,7 +7551,7 @@
       <c r="Q109" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="R109" s="5" t="s">
+      <c r="R109" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -7606,7 +7605,7 @@
       <c r="Q110" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="R110" s="5" t="s">
+      <c r="R110" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -7660,7 +7659,7 @@
       <c r="Q111" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="R111" s="5" t="s">
+      <c r="R111" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -7714,7 +7713,7 @@
       <c r="Q112" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="R112" s="5" t="s">
+      <c r="R112" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -7768,7 +7767,7 @@
       <c r="Q113" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="R113" s="5" t="s">
+      <c r="R113" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -7822,7 +7821,7 @@
       <c r="Q114" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="R114" s="5" t="s">
+      <c r="R114" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -7876,7 +7875,7 @@
       <c r="Q115" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="R115" s="5" t="s">
+      <c r="R115" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -7930,7 +7929,7 @@
       <c r="Q116" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="R116" s="5" t="s">
+      <c r="R116" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -7984,7 +7983,7 @@
       <c r="Q117" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="R117" s="5" t="s">
+      <c r="R117" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -8038,7 +8037,7 @@
       <c r="Q118" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="R118" s="5" t="s">
+      <c r="R118" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -8092,7 +8091,7 @@
       <c r="Q119" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="R119" s="5" t="s">
+      <c r="R119" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -8146,7 +8145,7 @@
       <c r="Q120" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="R120" s="5" t="s">
+      <c r="R120" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -8200,7 +8199,7 @@
       <c r="Q121" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="R121" s="5" t="s">
+      <c r="R121" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -8254,7 +8253,7 @@
       <c r="Q122" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="R122" s="5" t="s">
+      <c r="R122" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -8308,7 +8307,7 @@
       <c r="Q123" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="R123" s="5" t="s">
+      <c r="R123" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -8362,7 +8361,7 @@
       <c r="Q124" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="R124" s="5" t="s">
+      <c r="R124" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -8416,7 +8415,7 @@
       <c r="Q125" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="R125" s="5" t="s">
+      <c r="R125" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -8470,7 +8469,7 @@
       <c r="Q126" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="R126" s="5" t="s">
+      <c r="R126" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -8524,7 +8523,7 @@
       <c r="Q127" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="R127" s="5" t="s">
+      <c r="R127" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -8578,7 +8577,7 @@
       <c r="Q128" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="R128" s="5" t="s">
+      <c r="R128" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -8632,7 +8631,7 @@
       <c r="Q129" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="R129" s="5" t="s">
+      <c r="R129" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -8686,7 +8685,7 @@
       <c r="Q130" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="R130" s="5" t="s">
+      <c r="R130" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -8740,7 +8739,7 @@
       <c r="Q131" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="R131" s="5" t="s">
+      <c r="R131" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -8794,7 +8793,7 @@
       <c r="Q132" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="R132" s="5" t="s">
+      <c r="R132" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -8848,7 +8847,7 @@
       <c r="Q133" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="R133" s="5" t="s">
+      <c r="R133" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -8902,7 +8901,7 @@
       <c r="Q134" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="R134" s="5" t="s">
+      <c r="R134" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -8956,7 +8955,7 @@
       <c r="Q135" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="R135" s="5" t="s">
+      <c r="R135" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -9010,7 +9009,7 @@
       <c r="Q136" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="R136" s="5" t="s">
+      <c r="R136" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -9064,7 +9063,7 @@
       <c r="Q137" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="R137" s="5" t="s">
+      <c r="R137" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -9118,7 +9117,7 @@
       <c r="Q138" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="R138" s="5" t="s">
+      <c r="R138" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -9172,7 +9171,7 @@
       <c r="Q139" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="R139" s="5" t="s">
+      <c r="R139" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -9226,7 +9225,7 @@
       <c r="Q140" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="R140" s="5" t="s">
+      <c r="R140" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -9280,7 +9279,7 @@
       <c r="Q141" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="R141" s="5" t="s">
+      <c r="R141" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -9334,7 +9333,7 @@
       <c r="Q142" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="R142" s="5" t="s">
+      <c r="R142" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -9388,7 +9387,7 @@
       <c r="Q143" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="R143" s="5" t="s">
+      <c r="R143" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -9442,7 +9441,7 @@
       <c r="Q144" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="R144" s="5" t="s">
+      <c r="R144" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -9496,7 +9495,7 @@
       <c r="Q145" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="R145" s="5" t="s">
+      <c r="R145" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -9550,7 +9549,7 @@
       <c r="Q146" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="R146" s="5" t="s">
+      <c r="R146" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -9604,7 +9603,7 @@
       <c r="Q147" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="R147" s="5" t="s">
+      <c r="R147" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -9658,7 +9657,7 @@
       <c r="Q148" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="R148" s="5" t="s">
+      <c r="R148" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -9712,7 +9711,7 @@
       <c r="Q149" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="R149" s="5" t="s">
+      <c r="R149" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -9766,7 +9765,7 @@
       <c r="Q150" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="R150" s="5" t="s">
+      <c r="R150" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -9820,7 +9819,7 @@
       <c r="Q151" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="R151" s="5" t="s">
+      <c r="R151" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -9874,7 +9873,7 @@
       <c r="Q152" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="R152" s="5" t="s">
+      <c r="R152" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -9928,7 +9927,7 @@
       <c r="Q153" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="R153" s="5" t="s">
+      <c r="R153" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -9982,7 +9981,7 @@
       <c r="Q154" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="R154" s="5" t="s">
+      <c r="R154" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -10036,7 +10035,7 @@
       <c r="Q155" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="R155" s="5" t="s">
+      <c r="R155" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -10090,7 +10089,7 @@
       <c r="Q156" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="R156" s="5" t="s">
+      <c r="R156" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -10144,7 +10143,7 @@
       <c r="Q157" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="R157" s="5" t="s">
+      <c r="R157" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -10198,7 +10197,7 @@
       <c r="Q158" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="R158" s="5" t="s">
+      <c r="R158" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -10252,7 +10251,7 @@
       <c r="Q159" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="R159" s="5" t="s">
+      <c r="R159" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -10306,7 +10305,7 @@
       <c r="Q160" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="R160" s="5" t="s">
+      <c r="R160" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -10360,7 +10359,7 @@
       <c r="Q161" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="R161" s="5" t="s">
+      <c r="R161" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -10414,7 +10413,7 @@
       <c r="Q162" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="R162" s="5" t="s">
+      <c r="R162" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -10468,7 +10467,7 @@
       <c r="Q163" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="R163" s="5" t="s">
+      <c r="R163" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -10522,7 +10521,7 @@
       <c r="Q164" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="R164" s="5" t="s">
+      <c r="R164" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -10576,7 +10575,7 @@
       <c r="Q165" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="R165" s="5" t="s">
+      <c r="R165" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -10630,7 +10629,7 @@
       <c r="Q166" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="R166" s="5" t="s">
+      <c r="R166" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -10684,7 +10683,7 @@
       <c r="Q167" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="R167" s="5" t="s">
+      <c r="R167" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -10738,7 +10737,7 @@
       <c r="Q168" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="R168" s="5" t="s">
+      <c r="R168" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -10792,7 +10791,7 @@
       <c r="Q169" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="R169" s="5" t="s">
+      <c r="R169" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -10846,7 +10845,7 @@
       <c r="Q170" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="R170" s="5" t="s">
+      <c r="R170" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -10900,7 +10899,7 @@
       <c r="Q171" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="R171" s="5" t="s">
+      <c r="R171" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -10954,7 +10953,7 @@
       <c r="Q172" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="R172" s="5" t="s">
+      <c r="R172" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -11008,7 +11007,7 @@
       <c r="Q173" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="R173" s="5" t="s">
+      <c r="R173" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -11062,7 +11061,7 @@
       <c r="Q174" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="R174" s="5" t="s">
+      <c r="R174" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -11116,7 +11115,7 @@
       <c r="Q175" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="R175" s="5" t="s">
+      <c r="R175" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -11170,7 +11169,7 @@
       <c r="Q176" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="R176" s="5" t="s">
+      <c r="R176" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -11224,7 +11223,7 @@
       <c r="Q177" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="R177" s="5" t="s">
+      <c r="R177" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -11278,7 +11277,7 @@
       <c r="Q178" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="R178" s="5" t="s">
+      <c r="R178" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -11332,7 +11331,7 @@
       <c r="Q179" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="R179" s="5" t="s">
+      <c r="R179" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -11386,7 +11385,7 @@
       <c r="Q180" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="R180" s="5" t="s">
+      <c r="R180" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -11440,7 +11439,7 @@
       <c r="Q181" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="R181" s="5" t="s">
+      <c r="R181" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -11494,7 +11493,7 @@
       <c r="Q182" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="R182" s="5" t="s">
+      <c r="R182" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -11548,7 +11547,7 @@
       <c r="Q183" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="R183" s="5" t="s">
+      <c r="R183" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -11602,7 +11601,7 @@
       <c r="Q184" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="R184" s="5" t="s">
+      <c r="R184" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -11656,7 +11655,7 @@
       <c r="Q185" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="R185" s="5" t="s">
+      <c r="R185" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -11710,7 +11709,7 @@
       <c r="Q186" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="R186" s="5" t="s">
+      <c r="R186" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -11764,7 +11763,7 @@
       <c r="Q187" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="R187" s="5" t="s">
+      <c r="R187" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -11818,7 +11817,7 @@
       <c r="Q188" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="R188" s="5" t="s">
+      <c r="R188" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -11872,7 +11871,7 @@
       <c r="Q189" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="R189" s="5" t="s">
+      <c r="R189" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -11926,7 +11925,7 @@
       <c r="Q190" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="R190" s="5" t="s">
+      <c r="R190" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -11980,7 +11979,7 @@
       <c r="Q191" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="R191" s="5" t="s">
+      <c r="R191" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -12034,7 +12033,7 @@
       <c r="Q192" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="R192" s="5" t="s">
+      <c r="R192" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -12088,7 +12087,7 @@
       <c r="Q193" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="R193" s="5" t="s">
+      <c r="R193" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -12142,7 +12141,7 @@
       <c r="Q194" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="R194" s="5" t="s">
+      <c r="R194" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -12196,7 +12195,7 @@
       <c r="Q195" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="R195" s="5" t="s">
+      <c r="R195" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -12250,7 +12249,7 @@
       <c r="Q196" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="R196" s="5" t="s">
+      <c r="R196" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -12304,7 +12303,7 @@
       <c r="Q197" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="R197" s="5" t="s">
+      <c r="R197" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -12358,7 +12357,7 @@
       <c r="Q198" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="R198" s="5" t="s">
+      <c r="R198" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -12412,7 +12411,7 @@
       <c r="Q199" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="R199" s="5" t="s">
+      <c r="R199" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -12466,7 +12465,7 @@
       <c r="Q200" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="R200" s="5" t="s">
+      <c r="R200" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -12520,7 +12519,7 @@
       <c r="Q201" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="R201" s="5" t="s">
+      <c r="R201" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -12574,7 +12573,7 @@
       <c r="Q202" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="R202" s="5" t="s">
+      <c r="R202" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -12628,7 +12627,7 @@
       <c r="Q203" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="R203" s="5" t="s">
+      <c r="R203" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -12682,7 +12681,7 @@
       <c r="Q204" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="R204" s="5" t="s">
+      <c r="R204" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -12736,7 +12735,7 @@
       <c r="Q205" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="R205" s="5" t="s">
+      <c r="R205" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -12790,7 +12789,7 @@
       <c r="Q206" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="R206" s="5" t="s">
+      <c r="R206" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -12844,7 +12843,7 @@
       <c r="Q207" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="R207" s="5" t="s">
+      <c r="R207" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -12898,7 +12897,7 @@
       <c r="Q208" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="R208" s="5" t="s">
+      <c r="R208" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -12952,7 +12951,7 @@
       <c r="Q209" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="R209" s="5" t="s">
+      <c r="R209" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -13006,7 +13005,7 @@
       <c r="Q210" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="R210" s="5" t="s">
+      <c r="R210" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -13060,7 +13059,7 @@
       <c r="Q211" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="R211" s="5" t="s">
+      <c r="R211" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -13114,7 +13113,7 @@
       <c r="Q212" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="R212" s="5" t="s">
+      <c r="R212" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -13168,7 +13167,7 @@
       <c r="Q213" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="R213" s="5" t="s">
+      <c r="R213" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -13222,7 +13221,7 @@
       <c r="Q214" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="R214" s="5" t="s">
+      <c r="R214" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -13276,7 +13275,7 @@
       <c r="Q215" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="R215" s="5" t="s">
+      <c r="R215" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -13330,7 +13329,7 @@
       <c r="Q216" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="R216" s="5" t="s">
+      <c r="R216" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -13384,7 +13383,7 @@
       <c r="Q217" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="R217" s="5" t="s">
+      <c r="R217" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -13438,7 +13437,7 @@
       <c r="Q218" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="R218" s="5" t="s">
+      <c r="R218" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -13492,7 +13491,7 @@
       <c r="Q219" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="R219" s="5" t="s">
+      <c r="R219" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -13546,7 +13545,7 @@
       <c r="Q220" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="R220" s="5" t="s">
+      <c r="R220" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -13600,7 +13599,7 @@
       <c r="Q221" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="R221" s="5" t="s">
+      <c r="R221" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -13654,7 +13653,7 @@
       <c r="Q222" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="R222" s="5" t="s">
+      <c r="R222" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -13708,7 +13707,7 @@
       <c r="Q223" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="R223" s="5" t="s">
+      <c r="R223" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -13762,7 +13761,7 @@
       <c r="Q224" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="R224" s="5" t="s">
+      <c r="R224" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -13816,7 +13815,7 @@
       <c r="Q225" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="R225" s="5" t="s">
+      <c r="R225" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -13870,7 +13869,7 @@
       <c r="Q226" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="R226" s="5" t="s">
+      <c r="R226" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -13924,7 +13923,7 @@
       <c r="Q227" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="R227" s="5" t="s">
+      <c r="R227" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -13978,7 +13977,7 @@
       <c r="Q228" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="R228" s="5" t="s">
+      <c r="R228" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -14032,7 +14031,7 @@
       <c r="Q229" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="R229" s="5" t="s">
+      <c r="R229" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -14086,7 +14085,7 @@
       <c r="Q230" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="R230" s="5" t="s">
+      <c r="R230" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -14140,7 +14139,7 @@
       <c r="Q231" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="R231" s="5" t="s">
+      <c r="R231" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -14194,7 +14193,7 @@
       <c r="Q232" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="R232" s="5" t="s">
+      <c r="R232" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -14248,7 +14247,7 @@
       <c r="Q233" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="R233" s="5" t="s">
+      <c r="R233" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -14302,7 +14301,7 @@
       <c r="Q234" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="R234" s="5" t="s">
+      <c r="R234" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -14356,7 +14355,7 @@
       <c r="Q235" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="R235" s="5" t="s">
+      <c r="R235" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -14410,7 +14409,7 @@
       <c r="Q236" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="R236" s="5" t="s">
+      <c r="R236" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -14464,7 +14463,7 @@
       <c r="Q237" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="R237" s="5" t="s">
+      <c r="R237" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -14518,7 +14517,7 @@
       <c r="Q238" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="R238" s="5" t="s">
+      <c r="R238" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -14572,7 +14571,7 @@
       <c r="Q239" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="R239" s="5" t="s">
+      <c r="R239" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -14626,7 +14625,7 @@
       <c r="Q240" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="R240" s="5" t="s">
+      <c r="R240" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -14680,7 +14679,7 @@
       <c r="Q241" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="R241" s="5" t="s">
+      <c r="R241" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -14734,7 +14733,7 @@
       <c r="Q242" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="R242" s="5" t="s">
+      <c r="R242" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -14788,7 +14787,7 @@
       <c r="Q243" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="R243" s="5" t="s">
+      <c r="R243" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -14842,7 +14841,7 @@
       <c r="Q244" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="R244" s="5" t="s">
+      <c r="R244" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -14896,7 +14895,7 @@
       <c r="Q245" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="R245" s="5" t="s">
+      <c r="R245" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -14950,7 +14949,7 @@
       <c r="Q246" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="R246" s="5" t="s">
+      <c r="R246" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -15004,7 +15003,7 @@
       <c r="Q247" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="R247" s="5" t="s">
+      <c r="R247" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -15058,7 +15057,7 @@
       <c r="Q248" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="R248" s="5" t="s">
+      <c r="R248" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -15112,7 +15111,7 @@
       <c r="Q249" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="R249" s="5" t="s">
+      <c r="R249" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -15166,7 +15165,7 @@
       <c r="Q250" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="R250" s="5" t="s">
+      <c r="R250" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -15220,7 +15219,7 @@
       <c r="Q251" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="R251" s="5" t="s">
+      <c r="R251" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -15274,7 +15273,7 @@
       <c r="Q252" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="R252" s="5" t="s">
+      <c r="R252" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -15328,7 +15327,7 @@
       <c r="Q253" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="R253" s="5" t="s">
+      <c r="R253" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -15382,7 +15381,7 @@
       <c r="Q254" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="R254" s="5" t="s">
+      <c r="R254" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -15436,7 +15435,7 @@
       <c r="Q255" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="R255" s="5" t="s">
+      <c r="R255" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -15490,7 +15489,7 @@
       <c r="Q256" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="R256" s="5" t="s">
+      <c r="R256" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -15544,7 +15543,7 @@
       <c r="Q257" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="R257" s="5" t="s">
+      <c r="R257" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -15598,7 +15597,7 @@
       <c r="Q258" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="R258" s="5" t="s">
+      <c r="R258" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -15652,7 +15651,7 @@
       <c r="Q259" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="R259" s="5" t="s">
+      <c r="R259" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -15706,7 +15705,7 @@
       <c r="Q260" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="R260" s="5" t="s">
+      <c r="R260" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -15760,7 +15759,7 @@
       <c r="Q261" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="R261" s="5" t="s">
+      <c r="R261" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -15814,7 +15813,7 @@
       <c r="Q262" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="R262" s="5" t="s">
+      <c r="R262" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -15868,7 +15867,7 @@
       <c r="Q263" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="R263" s="5" t="s">
+      <c r="R263" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -15922,7 +15921,7 @@
       <c r="Q264" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="R264" s="5" t="s">
+      <c r="R264" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -15976,7 +15975,7 @@
       <c r="Q265" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="R265" s="5" t="s">
+      <c r="R265" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -16030,7 +16029,7 @@
       <c r="Q266" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="R266" s="5" t="s">
+      <c r="R266" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -16084,7 +16083,7 @@
       <c r="Q267" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="R267" s="5" t="s">
+      <c r="R267" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -16138,7 +16137,7 @@
       <c r="Q268" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="R268" s="5" t="s">
+      <c r="R268" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -16192,7 +16191,7 @@
       <c r="Q269" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="R269" s="5" t="s">
+      <c r="R269" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -16246,7 +16245,7 @@
       <c r="Q270" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="R270" s="5" t="s">
+      <c r="R270" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -16300,7 +16299,7 @@
       <c r="Q271" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="R271" s="5" t="s">
+      <c r="R271" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -16354,7 +16353,7 @@
       <c r="Q272" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="R272" s="5" t="s">
+      <c r="R272" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -16408,7 +16407,7 @@
       <c r="Q273" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="R273" s="5" t="s">
+      <c r="R273" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -16462,7 +16461,7 @@
       <c r="Q274" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="R274" s="5" t="s">
+      <c r="R274" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -16516,7 +16515,7 @@
       <c r="Q275" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="R275" s="5" t="s">
+      <c r="R275" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -16570,7 +16569,7 @@
       <c r="Q276" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="R276" s="5" t="s">
+      <c r="R276" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -16624,7 +16623,7 @@
       <c r="Q277" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="R277" s="5" t="s">
+      <c r="R277" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -16678,7 +16677,7 @@
       <c r="Q278" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="R278" s="5" t="s">
+      <c r="R278" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -16732,7 +16731,7 @@
       <c r="Q279" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="R279" s="5" t="s">
+      <c r="R279" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -16786,7 +16785,7 @@
       <c r="Q280" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="R280" s="5" t="s">
+      <c r="R280" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -16840,7 +16839,7 @@
       <c r="Q281" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="R281" s="5" t="s">
+      <c r="R281" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -16894,7 +16893,7 @@
       <c r="Q282" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="R282" s="5" t="s">
+      <c r="R282" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -16948,7 +16947,7 @@
       <c r="Q283" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="R283" s="5" t="s">
+      <c r="R283" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -17002,7 +17001,7 @@
       <c r="Q284" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="R284" s="5" t="s">
+      <c r="R284" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -17056,24 +17055,24 @@
       <c r="Q285" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="R285" s="5" t="s">
+      <c r="R285" s="2" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="287" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="E287" s="7" t="s">
+      <c r="E287" s="6" t="s">
         <v>198</v>
       </c>
-      <c r="F287" s="8">
+      <c r="F287" s="7">
         <f>SUMIF(Tabela1[repasse],TRUE,Tabela1[valor])</f>
         <v>651375.73</v>
       </c>
     </row>
     <row r="288" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="E288" s="7" t="s">
+      <c r="E288" s="6" t="s">
         <v>199</v>
       </c>
-      <c r="F288" s="8">
+      <c r="F288" s="7">
         <f>SUMIF(Tabela1[pj],TRUE,Tabela1[valor])</f>
         <v>0</v>
       </c>
@@ -17087,6 +17086,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101006C56FB2846673243A9735D5EC6051572" ma:contentTypeVersion="11" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="36569ac63cfce8ff0f8884bc80e67f1c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5a5f483f-f768-438e-b4ef-63f46a7558dd" xmlns:ns3="dd8c73df-45bd-468c-aae5-f3faedcbd5e2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2040da04b75a9ea4fe796fa8180f8ca6" ns2:_="" ns3:_="">
     <xsd:import namespace="5a5f483f-f768-438e-b4ef-63f46a7558dd"/>
@@ -17281,15 +17289,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -17302,13 +17301,39 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B5FA29D8-99F9-4C82-862C-25403C7D3E2F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C47772C-3A10-4024-AA63-4DEDA8BCEC6F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C47772C-3A10-4024-AA63-4DEDA8BCEC6F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B5FA29D8-99F9-4C82-862C-25403C7D3E2F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="5a5f483f-f768-438e-b4ef-63f46a7558dd"/>
+    <ds:schemaRef ds:uri="dd8c73df-45bd-468c-aae5-f3faedcbd5e2"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{448E610F-7542-4F66-9968-C8F017F22501}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{448E610F-7542-4F66-9968-C8F017F22501}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="5a5f483f-f768-438e-b4ef-63f46a7558dd"/>
+    <ds:schemaRef ds:uri="dd8c73df-45bd-468c-aae5-f3faedcbd5e2"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>